<commit_message>
fix(hr): fit sample job levels to their column; patch npm advisories
- The sample job levels "Üst Yönetici" and "Uzman Yardımcısı" exceeded the
  10 character limit; a unit test now checks every sample cell against
  its column's maximum length
- npm audit fix (fast-uri, zod, orval 8.44.0) and an override of undici
  7.30.1 for @scalar/json-magic 0.15.7, which orval still pins

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/1-unvanlar.xlsx
+++ b/samples/1-unvanlar.xlsx
@@ -37,7 +37,7 @@
     <x:t>Yönetim</x:t>
   </x:si>
   <x:si>
-    <x:t>Üst Yönetici</x:t>
+    <x:t>Yönetici</x:t>
   </x:si>
   <x:si>
     <x:t>DIR</x:t>
@@ -142,7 +142,7 @@
     <x:t>Destek Uzmanı</x:t>
   </x:si>
   <x:si>
-    <x:t>Uzman Yardımcısı</x:t>
+    <x:t>Yardımcı</x:t>
   </x:si>
   <x:si>
     <x:t>URT-OPR</x:t>
@@ -589,7 +589,7 @@
     <x:col min="1" max="1" width="13.424911" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="22.996339" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="15.853482" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="9.853482" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4">

</xml_diff>